<commit_message>
Fix staff-phone alert, newsletter image prompt; rebuild grading (CA 30 + Exam 70, JSS/SSS scales)
- Dashboard: "no phone number" now counts only teachers listed on the Teachers
  page; the seeded admin account no longer creates a phantom alert.
- Classes & Arms: placeholder SS4 -> JSS3.
- Newsletter posts no longer ask for or store a picture (blog only), enforced
  in the editor and on the server.
- Grading: CA 30 (10+2+3, 10+3+2) + Exam 70. Senior classes use WAEC A1-F9,
  junior classes use A/C/P/F. results.is_junior records the scale per result
  so promoted students keep earlier grades. Excel template, importer, OCR
  limits, sheets, report cards and dashboards updated.
- database/007_grading_30_70.sql migration (idempotent, keeps existing marks),
  folded into schema.sql. Added scheme unit tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LGBC8VLeJ1KVwH9EQdxGNr
</commit_message>
<xml_diff>
--- a/score-sheet-template.xlsx
+++ b/score-sheet-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>NIGERIAN NAVY SECONDARY SCHOOL AKPABUYO CALABAR</t>
   </si>
@@ -34,6 +34,12 @@
     <t>FORM TEACHER:</t>
   </si>
   <si>
+    <t>LEVEL:</t>
+  </si>
+  <si>
+    <t>SSS</t>
+  </si>
+  <si>
     <t>NO IN CLASS:</t>
   </si>
   <si>
@@ -43,7 +49,7 @@
     <t>SUBJECT:</t>
   </si>
   <si>
-    <t>Fill the yellow cells only (leave a row blank for a student who sat nothing). Student ID is optional - if it is left blank the importer matches by name. Totals and grade calculate themselves.</t>
+    <t>Fill the yellow cells only (leave a row blank for a student who sat nothing). Student ID is optional - if it is left blank the importer matches by name. Totals and grade calculate themselves (choose JSS or SSS in the LEVEL box so the right grading scale is used).</t>
   </si>
   <si>
     <t>S/NO</t>
@@ -55,31 +61,31 @@
     <t>STUDENTS NAME</t>
   </si>
   <si>
-    <t>1ST TEST (15%)</t>
-  </si>
-  <si>
-    <t>QUIZ (5%)</t>
-  </si>
-  <si>
-    <t>ASSIGNMENT (5%)</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>2ND TEST (5%)</t>
-  </si>
-  <si>
-    <t>PROJECT (5%)</t>
-  </si>
-  <si>
-    <t>NOTE (5%)</t>
-  </si>
-  <si>
-    <t>EXAM (60%)</t>
-  </si>
-  <si>
-    <t>TERM'S TOTAL</t>
+    <t>1ST TEST (10)</t>
+  </si>
+  <si>
+    <t>QUIZ (2)</t>
+  </si>
+  <si>
+    <t>ASSIGNMENT (3)</t>
+  </si>
+  <si>
+    <t>TOTAL (15)</t>
+  </si>
+  <si>
+    <t>2ND TEST (10)</t>
+  </si>
+  <si>
+    <t>PROJECT (3)</t>
+  </si>
+  <si>
+    <t>NOTE (2)</t>
+  </si>
+  <si>
+    <t>EXAM (70)</t>
+  </si>
+  <si>
+    <t>TERM'S TOTAL (100)</t>
   </si>
   <si>
     <t>GRADE</t>
@@ -626,20 +632,24 @@
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
+      <c r="L3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>3</v>
@@ -647,7 +657,7 @@
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>3</v>
@@ -660,7 +670,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -678,46 +688,46 @@
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>16</v>
-      </c>
       <c r="L6" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -743,7 +753,7 @@
         <f>IF(COUNT(D7:J7,L7)=0,"",SUM(G7,K7,L7))</f>
       </c>
       <c r="N7" s="11">
-        <f>IF(M7="","",IF(M7&gt;=75,"A1",IF(M7&gt;=70,"B2",IF(M7&gt;=65,"B3",IF(M7&gt;=60,"C4",IF(M7&gt;=55,"C5",IF(M7&gt;=50,"C6",IF(M7&gt;=45,"D7",IF(M7&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M7="","",IF($M$3="JSS",IF(M7&gt;=80,"A",IF(M7&gt;=60,"C",IF(M7&gt;=50,"P","F"))),IF(M7&gt;=75,"A1",IF(M7&gt;=70,"B2",IF(M7&gt;=65,"B3",IF(M7&gt;=60,"C4",IF(M7&gt;=55,"C5",IF(M7&gt;=50,"C6",IF(M7&gt;=45,"D7",IF(M7&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -769,7 +779,7 @@
         <f>IF(COUNT(D8:J8,L8)=0,"",SUM(G8,K8,L8))</f>
       </c>
       <c r="N8" s="11">
-        <f>IF(M8="","",IF(M8&gt;=75,"A1",IF(M8&gt;=70,"B2",IF(M8&gt;=65,"B3",IF(M8&gt;=60,"C4",IF(M8&gt;=55,"C5",IF(M8&gt;=50,"C6",IF(M8&gt;=45,"D7",IF(M8&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M8="","",IF($M$3="JSS",IF(M8&gt;=80,"A",IF(M8&gt;=60,"C",IF(M8&gt;=50,"P","F"))),IF(M8&gt;=75,"A1",IF(M8&gt;=70,"B2",IF(M8&gt;=65,"B3",IF(M8&gt;=60,"C4",IF(M8&gt;=55,"C5",IF(M8&gt;=50,"C6",IF(M8&gt;=45,"D7",IF(M8&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -795,7 +805,7 @@
         <f>IF(COUNT(D9:J9,L9)=0,"",SUM(G9,K9,L9))</f>
       </c>
       <c r="N9" s="11">
-        <f>IF(M9="","",IF(M9&gt;=75,"A1",IF(M9&gt;=70,"B2",IF(M9&gt;=65,"B3",IF(M9&gt;=60,"C4",IF(M9&gt;=55,"C5",IF(M9&gt;=50,"C6",IF(M9&gt;=45,"D7",IF(M9&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M9="","",IF($M$3="JSS",IF(M9&gt;=80,"A",IF(M9&gt;=60,"C",IF(M9&gt;=50,"P","F"))),IF(M9&gt;=75,"A1",IF(M9&gt;=70,"B2",IF(M9&gt;=65,"B3",IF(M9&gt;=60,"C4",IF(M9&gt;=55,"C5",IF(M9&gt;=50,"C6",IF(M9&gt;=45,"D7",IF(M9&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -821,7 +831,7 @@
         <f>IF(COUNT(D10:J10,L10)=0,"",SUM(G10,K10,L10))</f>
       </c>
       <c r="N10" s="11">
-        <f>IF(M10="","",IF(M10&gt;=75,"A1",IF(M10&gt;=70,"B2",IF(M10&gt;=65,"B3",IF(M10&gt;=60,"C4",IF(M10&gt;=55,"C5",IF(M10&gt;=50,"C6",IF(M10&gt;=45,"D7",IF(M10&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M10="","",IF($M$3="JSS",IF(M10&gt;=80,"A",IF(M10&gt;=60,"C",IF(M10&gt;=50,"P","F"))),IF(M10&gt;=75,"A1",IF(M10&gt;=70,"B2",IF(M10&gt;=65,"B3",IF(M10&gt;=60,"C4",IF(M10&gt;=55,"C5",IF(M10&gt;=50,"C6",IF(M10&gt;=45,"D7",IF(M10&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -847,7 +857,7 @@
         <f>IF(COUNT(D11:J11,L11)=0,"",SUM(G11,K11,L11))</f>
       </c>
       <c r="N11" s="11">
-        <f>IF(M11="","",IF(M11&gt;=75,"A1",IF(M11&gt;=70,"B2",IF(M11&gt;=65,"B3",IF(M11&gt;=60,"C4",IF(M11&gt;=55,"C5",IF(M11&gt;=50,"C6",IF(M11&gt;=45,"D7",IF(M11&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M11="","",IF($M$3="JSS",IF(M11&gt;=80,"A",IF(M11&gt;=60,"C",IF(M11&gt;=50,"P","F"))),IF(M11&gt;=75,"A1",IF(M11&gt;=70,"B2",IF(M11&gt;=65,"B3",IF(M11&gt;=60,"C4",IF(M11&gt;=55,"C5",IF(M11&gt;=50,"C6",IF(M11&gt;=45,"D7",IF(M11&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -873,7 +883,7 @@
         <f>IF(COUNT(D12:J12,L12)=0,"",SUM(G12,K12,L12))</f>
       </c>
       <c r="N12" s="11">
-        <f>IF(M12="","",IF(M12&gt;=75,"A1",IF(M12&gt;=70,"B2",IF(M12&gt;=65,"B3",IF(M12&gt;=60,"C4",IF(M12&gt;=55,"C5",IF(M12&gt;=50,"C6",IF(M12&gt;=45,"D7",IF(M12&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M12="","",IF($M$3="JSS",IF(M12&gt;=80,"A",IF(M12&gt;=60,"C",IF(M12&gt;=50,"P","F"))),IF(M12&gt;=75,"A1",IF(M12&gt;=70,"B2",IF(M12&gt;=65,"B3",IF(M12&gt;=60,"C4",IF(M12&gt;=55,"C5",IF(M12&gt;=50,"C6",IF(M12&gt;=45,"D7",IF(M12&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -899,7 +909,7 @@
         <f>IF(COUNT(D13:J13,L13)=0,"",SUM(G13,K13,L13))</f>
       </c>
       <c r="N13" s="11">
-        <f>IF(M13="","",IF(M13&gt;=75,"A1",IF(M13&gt;=70,"B2",IF(M13&gt;=65,"B3",IF(M13&gt;=60,"C4",IF(M13&gt;=55,"C5",IF(M13&gt;=50,"C6",IF(M13&gt;=45,"D7",IF(M13&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M13="","",IF($M$3="JSS",IF(M13&gt;=80,"A",IF(M13&gt;=60,"C",IF(M13&gt;=50,"P","F"))),IF(M13&gt;=75,"A1",IF(M13&gt;=70,"B2",IF(M13&gt;=65,"B3",IF(M13&gt;=60,"C4",IF(M13&gt;=55,"C5",IF(M13&gt;=50,"C6",IF(M13&gt;=45,"D7",IF(M13&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -925,7 +935,7 @@
         <f>IF(COUNT(D14:J14,L14)=0,"",SUM(G14,K14,L14))</f>
       </c>
       <c r="N14" s="11">
-        <f>IF(M14="","",IF(M14&gt;=75,"A1",IF(M14&gt;=70,"B2",IF(M14&gt;=65,"B3",IF(M14&gt;=60,"C4",IF(M14&gt;=55,"C5",IF(M14&gt;=50,"C6",IF(M14&gt;=45,"D7",IF(M14&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M14="","",IF($M$3="JSS",IF(M14&gt;=80,"A",IF(M14&gt;=60,"C",IF(M14&gt;=50,"P","F"))),IF(M14&gt;=75,"A1",IF(M14&gt;=70,"B2",IF(M14&gt;=65,"B3",IF(M14&gt;=60,"C4",IF(M14&gt;=55,"C5",IF(M14&gt;=50,"C6",IF(M14&gt;=45,"D7",IF(M14&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -951,7 +961,7 @@
         <f>IF(COUNT(D15:J15,L15)=0,"",SUM(G15,K15,L15))</f>
       </c>
       <c r="N15" s="11">
-        <f>IF(M15="","",IF(M15&gt;=75,"A1",IF(M15&gt;=70,"B2",IF(M15&gt;=65,"B3",IF(M15&gt;=60,"C4",IF(M15&gt;=55,"C5",IF(M15&gt;=50,"C6",IF(M15&gt;=45,"D7",IF(M15&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M15="","",IF($M$3="JSS",IF(M15&gt;=80,"A",IF(M15&gt;=60,"C",IF(M15&gt;=50,"P","F"))),IF(M15&gt;=75,"A1",IF(M15&gt;=70,"B2",IF(M15&gt;=65,"B3",IF(M15&gt;=60,"C4",IF(M15&gt;=55,"C5",IF(M15&gt;=50,"C6",IF(M15&gt;=45,"D7",IF(M15&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -977,7 +987,7 @@
         <f>IF(COUNT(D16:J16,L16)=0,"",SUM(G16,K16,L16))</f>
       </c>
       <c r="N16" s="11">
-        <f>IF(M16="","",IF(M16&gt;=75,"A1",IF(M16&gt;=70,"B2",IF(M16&gt;=65,"B3",IF(M16&gt;=60,"C4",IF(M16&gt;=55,"C5",IF(M16&gt;=50,"C6",IF(M16&gt;=45,"D7",IF(M16&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M16="","",IF($M$3="JSS",IF(M16&gt;=80,"A",IF(M16&gt;=60,"C",IF(M16&gt;=50,"P","F"))),IF(M16&gt;=75,"A1",IF(M16&gt;=70,"B2",IF(M16&gt;=65,"B3",IF(M16&gt;=60,"C4",IF(M16&gt;=55,"C5",IF(M16&gt;=50,"C6",IF(M16&gt;=45,"D7",IF(M16&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1003,7 +1013,7 @@
         <f>IF(COUNT(D17:J17,L17)=0,"",SUM(G17,K17,L17))</f>
       </c>
       <c r="N17" s="11">
-        <f>IF(M17="","",IF(M17&gt;=75,"A1",IF(M17&gt;=70,"B2",IF(M17&gt;=65,"B3",IF(M17&gt;=60,"C4",IF(M17&gt;=55,"C5",IF(M17&gt;=50,"C6",IF(M17&gt;=45,"D7",IF(M17&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M17="","",IF($M$3="JSS",IF(M17&gt;=80,"A",IF(M17&gt;=60,"C",IF(M17&gt;=50,"P","F"))),IF(M17&gt;=75,"A1",IF(M17&gt;=70,"B2",IF(M17&gt;=65,"B3",IF(M17&gt;=60,"C4",IF(M17&gt;=55,"C5",IF(M17&gt;=50,"C6",IF(M17&gt;=45,"D7",IF(M17&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1029,7 +1039,7 @@
         <f>IF(COUNT(D18:J18,L18)=0,"",SUM(G18,K18,L18))</f>
       </c>
       <c r="N18" s="11">
-        <f>IF(M18="","",IF(M18&gt;=75,"A1",IF(M18&gt;=70,"B2",IF(M18&gt;=65,"B3",IF(M18&gt;=60,"C4",IF(M18&gt;=55,"C5",IF(M18&gt;=50,"C6",IF(M18&gt;=45,"D7",IF(M18&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M18="","",IF($M$3="JSS",IF(M18&gt;=80,"A",IF(M18&gt;=60,"C",IF(M18&gt;=50,"P","F"))),IF(M18&gt;=75,"A1",IF(M18&gt;=70,"B2",IF(M18&gt;=65,"B3",IF(M18&gt;=60,"C4",IF(M18&gt;=55,"C5",IF(M18&gt;=50,"C6",IF(M18&gt;=45,"D7",IF(M18&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1055,7 +1065,7 @@
         <f>IF(COUNT(D19:J19,L19)=0,"",SUM(G19,K19,L19))</f>
       </c>
       <c r="N19" s="11">
-        <f>IF(M19="","",IF(M19&gt;=75,"A1",IF(M19&gt;=70,"B2",IF(M19&gt;=65,"B3",IF(M19&gt;=60,"C4",IF(M19&gt;=55,"C5",IF(M19&gt;=50,"C6",IF(M19&gt;=45,"D7",IF(M19&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M19="","",IF($M$3="JSS",IF(M19&gt;=80,"A",IF(M19&gt;=60,"C",IF(M19&gt;=50,"P","F"))),IF(M19&gt;=75,"A1",IF(M19&gt;=70,"B2",IF(M19&gt;=65,"B3",IF(M19&gt;=60,"C4",IF(M19&gt;=55,"C5",IF(M19&gt;=50,"C6",IF(M19&gt;=45,"D7",IF(M19&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1081,7 +1091,7 @@
         <f>IF(COUNT(D20:J20,L20)=0,"",SUM(G20,K20,L20))</f>
       </c>
       <c r="N20" s="11">
-        <f>IF(M20="","",IF(M20&gt;=75,"A1",IF(M20&gt;=70,"B2",IF(M20&gt;=65,"B3",IF(M20&gt;=60,"C4",IF(M20&gt;=55,"C5",IF(M20&gt;=50,"C6",IF(M20&gt;=45,"D7",IF(M20&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M20="","",IF($M$3="JSS",IF(M20&gt;=80,"A",IF(M20&gt;=60,"C",IF(M20&gt;=50,"P","F"))),IF(M20&gt;=75,"A1",IF(M20&gt;=70,"B2",IF(M20&gt;=65,"B3",IF(M20&gt;=60,"C4",IF(M20&gt;=55,"C5",IF(M20&gt;=50,"C6",IF(M20&gt;=45,"D7",IF(M20&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1107,7 +1117,7 @@
         <f>IF(COUNT(D21:J21,L21)=0,"",SUM(G21,K21,L21))</f>
       </c>
       <c r="N21" s="11">
-        <f>IF(M21="","",IF(M21&gt;=75,"A1",IF(M21&gt;=70,"B2",IF(M21&gt;=65,"B3",IF(M21&gt;=60,"C4",IF(M21&gt;=55,"C5",IF(M21&gt;=50,"C6",IF(M21&gt;=45,"D7",IF(M21&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M21="","",IF($M$3="JSS",IF(M21&gt;=80,"A",IF(M21&gt;=60,"C",IF(M21&gt;=50,"P","F"))),IF(M21&gt;=75,"A1",IF(M21&gt;=70,"B2",IF(M21&gt;=65,"B3",IF(M21&gt;=60,"C4",IF(M21&gt;=55,"C5",IF(M21&gt;=50,"C6",IF(M21&gt;=45,"D7",IF(M21&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1133,7 +1143,7 @@
         <f>IF(COUNT(D22:J22,L22)=0,"",SUM(G22,K22,L22))</f>
       </c>
       <c r="N22" s="11">
-        <f>IF(M22="","",IF(M22&gt;=75,"A1",IF(M22&gt;=70,"B2",IF(M22&gt;=65,"B3",IF(M22&gt;=60,"C4",IF(M22&gt;=55,"C5",IF(M22&gt;=50,"C6",IF(M22&gt;=45,"D7",IF(M22&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M22="","",IF($M$3="JSS",IF(M22&gt;=80,"A",IF(M22&gt;=60,"C",IF(M22&gt;=50,"P","F"))),IF(M22&gt;=75,"A1",IF(M22&gt;=70,"B2",IF(M22&gt;=65,"B3",IF(M22&gt;=60,"C4",IF(M22&gt;=55,"C5",IF(M22&gt;=50,"C6",IF(M22&gt;=45,"D7",IF(M22&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1159,7 +1169,7 @@
         <f>IF(COUNT(D23:J23,L23)=0,"",SUM(G23,K23,L23))</f>
       </c>
       <c r="N23" s="11">
-        <f>IF(M23="","",IF(M23&gt;=75,"A1",IF(M23&gt;=70,"B2",IF(M23&gt;=65,"B3",IF(M23&gt;=60,"C4",IF(M23&gt;=55,"C5",IF(M23&gt;=50,"C6",IF(M23&gt;=45,"D7",IF(M23&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M23="","",IF($M$3="JSS",IF(M23&gt;=80,"A",IF(M23&gt;=60,"C",IF(M23&gt;=50,"P","F"))),IF(M23&gt;=75,"A1",IF(M23&gt;=70,"B2",IF(M23&gt;=65,"B3",IF(M23&gt;=60,"C4",IF(M23&gt;=55,"C5",IF(M23&gt;=50,"C6",IF(M23&gt;=45,"D7",IF(M23&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1185,7 +1195,7 @@
         <f>IF(COUNT(D24:J24,L24)=0,"",SUM(G24,K24,L24))</f>
       </c>
       <c r="N24" s="11">
-        <f>IF(M24="","",IF(M24&gt;=75,"A1",IF(M24&gt;=70,"B2",IF(M24&gt;=65,"B3",IF(M24&gt;=60,"C4",IF(M24&gt;=55,"C5",IF(M24&gt;=50,"C6",IF(M24&gt;=45,"D7",IF(M24&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M24="","",IF($M$3="JSS",IF(M24&gt;=80,"A",IF(M24&gt;=60,"C",IF(M24&gt;=50,"P","F"))),IF(M24&gt;=75,"A1",IF(M24&gt;=70,"B2",IF(M24&gt;=65,"B3",IF(M24&gt;=60,"C4",IF(M24&gt;=55,"C5",IF(M24&gt;=50,"C6",IF(M24&gt;=45,"D7",IF(M24&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1211,7 +1221,7 @@
         <f>IF(COUNT(D25:J25,L25)=0,"",SUM(G25,K25,L25))</f>
       </c>
       <c r="N25" s="11">
-        <f>IF(M25="","",IF(M25&gt;=75,"A1",IF(M25&gt;=70,"B2",IF(M25&gt;=65,"B3",IF(M25&gt;=60,"C4",IF(M25&gt;=55,"C5",IF(M25&gt;=50,"C6",IF(M25&gt;=45,"D7",IF(M25&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M25="","",IF($M$3="JSS",IF(M25&gt;=80,"A",IF(M25&gt;=60,"C",IF(M25&gt;=50,"P","F"))),IF(M25&gt;=75,"A1",IF(M25&gt;=70,"B2",IF(M25&gt;=65,"B3",IF(M25&gt;=60,"C4",IF(M25&gt;=55,"C5",IF(M25&gt;=50,"C6",IF(M25&gt;=45,"D7",IF(M25&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1237,7 +1247,7 @@
         <f>IF(COUNT(D26:J26,L26)=0,"",SUM(G26,K26,L26))</f>
       </c>
       <c r="N26" s="11">
-        <f>IF(M26="","",IF(M26&gt;=75,"A1",IF(M26&gt;=70,"B2",IF(M26&gt;=65,"B3",IF(M26&gt;=60,"C4",IF(M26&gt;=55,"C5",IF(M26&gt;=50,"C6",IF(M26&gt;=45,"D7",IF(M26&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M26="","",IF($M$3="JSS",IF(M26&gt;=80,"A",IF(M26&gt;=60,"C",IF(M26&gt;=50,"P","F"))),IF(M26&gt;=75,"A1",IF(M26&gt;=70,"B2",IF(M26&gt;=65,"B3",IF(M26&gt;=60,"C4",IF(M26&gt;=55,"C5",IF(M26&gt;=50,"C6",IF(M26&gt;=45,"D7",IF(M26&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1263,7 +1273,7 @@
         <f>IF(COUNT(D27:J27,L27)=0,"",SUM(G27,K27,L27))</f>
       </c>
       <c r="N27" s="11">
-        <f>IF(M27="","",IF(M27&gt;=75,"A1",IF(M27&gt;=70,"B2",IF(M27&gt;=65,"B3",IF(M27&gt;=60,"C4",IF(M27&gt;=55,"C5",IF(M27&gt;=50,"C6",IF(M27&gt;=45,"D7",IF(M27&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M27="","",IF($M$3="JSS",IF(M27&gt;=80,"A",IF(M27&gt;=60,"C",IF(M27&gt;=50,"P","F"))),IF(M27&gt;=75,"A1",IF(M27&gt;=70,"B2",IF(M27&gt;=65,"B3",IF(M27&gt;=60,"C4",IF(M27&gt;=55,"C5",IF(M27&gt;=50,"C6",IF(M27&gt;=45,"D7",IF(M27&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1289,7 +1299,7 @@
         <f>IF(COUNT(D28:J28,L28)=0,"",SUM(G28,K28,L28))</f>
       </c>
       <c r="N28" s="11">
-        <f>IF(M28="","",IF(M28&gt;=75,"A1",IF(M28&gt;=70,"B2",IF(M28&gt;=65,"B3",IF(M28&gt;=60,"C4",IF(M28&gt;=55,"C5",IF(M28&gt;=50,"C6",IF(M28&gt;=45,"D7",IF(M28&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M28="","",IF($M$3="JSS",IF(M28&gt;=80,"A",IF(M28&gt;=60,"C",IF(M28&gt;=50,"P","F"))),IF(M28&gt;=75,"A1",IF(M28&gt;=70,"B2",IF(M28&gt;=65,"B3",IF(M28&gt;=60,"C4",IF(M28&gt;=55,"C5",IF(M28&gt;=50,"C6",IF(M28&gt;=45,"D7",IF(M28&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1315,7 +1325,7 @@
         <f>IF(COUNT(D29:J29,L29)=0,"",SUM(G29,K29,L29))</f>
       </c>
       <c r="N29" s="11">
-        <f>IF(M29="","",IF(M29&gt;=75,"A1",IF(M29&gt;=70,"B2",IF(M29&gt;=65,"B3",IF(M29&gt;=60,"C4",IF(M29&gt;=55,"C5",IF(M29&gt;=50,"C6",IF(M29&gt;=45,"D7",IF(M29&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M29="","",IF($M$3="JSS",IF(M29&gt;=80,"A",IF(M29&gt;=60,"C",IF(M29&gt;=50,"P","F"))),IF(M29&gt;=75,"A1",IF(M29&gt;=70,"B2",IF(M29&gt;=65,"B3",IF(M29&gt;=60,"C4",IF(M29&gt;=55,"C5",IF(M29&gt;=50,"C6",IF(M29&gt;=45,"D7",IF(M29&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1341,7 +1351,7 @@
         <f>IF(COUNT(D30:J30,L30)=0,"",SUM(G30,K30,L30))</f>
       </c>
       <c r="N30" s="11">
-        <f>IF(M30="","",IF(M30&gt;=75,"A1",IF(M30&gt;=70,"B2",IF(M30&gt;=65,"B3",IF(M30&gt;=60,"C4",IF(M30&gt;=55,"C5",IF(M30&gt;=50,"C6",IF(M30&gt;=45,"D7",IF(M30&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M30="","",IF($M$3="JSS",IF(M30&gt;=80,"A",IF(M30&gt;=60,"C",IF(M30&gt;=50,"P","F"))),IF(M30&gt;=75,"A1",IF(M30&gt;=70,"B2",IF(M30&gt;=65,"B3",IF(M30&gt;=60,"C4",IF(M30&gt;=55,"C5",IF(M30&gt;=50,"C6",IF(M30&gt;=45,"D7",IF(M30&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1367,7 +1377,7 @@
         <f>IF(COUNT(D31:J31,L31)=0,"",SUM(G31,K31,L31))</f>
       </c>
       <c r="N31" s="11">
-        <f>IF(M31="","",IF(M31&gt;=75,"A1",IF(M31&gt;=70,"B2",IF(M31&gt;=65,"B3",IF(M31&gt;=60,"C4",IF(M31&gt;=55,"C5",IF(M31&gt;=50,"C6",IF(M31&gt;=45,"D7",IF(M31&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M31="","",IF($M$3="JSS",IF(M31&gt;=80,"A",IF(M31&gt;=60,"C",IF(M31&gt;=50,"P","F"))),IF(M31&gt;=75,"A1",IF(M31&gt;=70,"B2",IF(M31&gt;=65,"B3",IF(M31&gt;=60,"C4",IF(M31&gt;=55,"C5",IF(M31&gt;=50,"C6",IF(M31&gt;=45,"D7",IF(M31&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1393,7 +1403,7 @@
         <f>IF(COUNT(D32:J32,L32)=0,"",SUM(G32,K32,L32))</f>
       </c>
       <c r="N32" s="11">
-        <f>IF(M32="","",IF(M32&gt;=75,"A1",IF(M32&gt;=70,"B2",IF(M32&gt;=65,"B3",IF(M32&gt;=60,"C4",IF(M32&gt;=55,"C5",IF(M32&gt;=50,"C6",IF(M32&gt;=45,"D7",IF(M32&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M32="","",IF($M$3="JSS",IF(M32&gt;=80,"A",IF(M32&gt;=60,"C",IF(M32&gt;=50,"P","F"))),IF(M32&gt;=75,"A1",IF(M32&gt;=70,"B2",IF(M32&gt;=65,"B3",IF(M32&gt;=60,"C4",IF(M32&gt;=55,"C5",IF(M32&gt;=50,"C6",IF(M32&gt;=45,"D7",IF(M32&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1419,7 +1429,7 @@
         <f>IF(COUNT(D33:J33,L33)=0,"",SUM(G33,K33,L33))</f>
       </c>
       <c r="N33" s="11">
-        <f>IF(M33="","",IF(M33&gt;=75,"A1",IF(M33&gt;=70,"B2",IF(M33&gt;=65,"B3",IF(M33&gt;=60,"C4",IF(M33&gt;=55,"C5",IF(M33&gt;=50,"C6",IF(M33&gt;=45,"D7",IF(M33&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M33="","",IF($M$3="JSS",IF(M33&gt;=80,"A",IF(M33&gt;=60,"C",IF(M33&gt;=50,"P","F"))),IF(M33&gt;=75,"A1",IF(M33&gt;=70,"B2",IF(M33&gt;=65,"B3",IF(M33&gt;=60,"C4",IF(M33&gt;=55,"C5",IF(M33&gt;=50,"C6",IF(M33&gt;=45,"D7",IF(M33&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1445,7 +1455,7 @@
         <f>IF(COUNT(D34:J34,L34)=0,"",SUM(G34,K34,L34))</f>
       </c>
       <c r="N34" s="11">
-        <f>IF(M34="","",IF(M34&gt;=75,"A1",IF(M34&gt;=70,"B2",IF(M34&gt;=65,"B3",IF(M34&gt;=60,"C4",IF(M34&gt;=55,"C5",IF(M34&gt;=50,"C6",IF(M34&gt;=45,"D7",IF(M34&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M34="","",IF($M$3="JSS",IF(M34&gt;=80,"A",IF(M34&gt;=60,"C",IF(M34&gt;=50,"P","F"))),IF(M34&gt;=75,"A1",IF(M34&gt;=70,"B2",IF(M34&gt;=65,"B3",IF(M34&gt;=60,"C4",IF(M34&gt;=55,"C5",IF(M34&gt;=50,"C6",IF(M34&gt;=45,"D7",IF(M34&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1471,7 +1481,7 @@
         <f>IF(COUNT(D35:J35,L35)=0,"",SUM(G35,K35,L35))</f>
       </c>
       <c r="N35" s="11">
-        <f>IF(M35="","",IF(M35&gt;=75,"A1",IF(M35&gt;=70,"B2",IF(M35&gt;=65,"B3",IF(M35&gt;=60,"C4",IF(M35&gt;=55,"C5",IF(M35&gt;=50,"C6",IF(M35&gt;=45,"D7",IF(M35&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M35="","",IF($M$3="JSS",IF(M35&gt;=80,"A",IF(M35&gt;=60,"C",IF(M35&gt;=50,"P","F"))),IF(M35&gt;=75,"A1",IF(M35&gt;=70,"B2",IF(M35&gt;=65,"B3",IF(M35&gt;=60,"C4",IF(M35&gt;=55,"C5",IF(M35&gt;=50,"C6",IF(M35&gt;=45,"D7",IF(M35&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1497,7 +1507,7 @@
         <f>IF(COUNT(D36:J36,L36)=0,"",SUM(G36,K36,L36))</f>
       </c>
       <c r="N36" s="11">
-        <f>IF(M36="","",IF(M36&gt;=75,"A1",IF(M36&gt;=70,"B2",IF(M36&gt;=65,"B3",IF(M36&gt;=60,"C4",IF(M36&gt;=55,"C5",IF(M36&gt;=50,"C6",IF(M36&gt;=45,"D7",IF(M36&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M36="","",IF($M$3="JSS",IF(M36&gt;=80,"A",IF(M36&gt;=60,"C",IF(M36&gt;=50,"P","F"))),IF(M36&gt;=75,"A1",IF(M36&gt;=70,"B2",IF(M36&gt;=65,"B3",IF(M36&gt;=60,"C4",IF(M36&gt;=55,"C5",IF(M36&gt;=50,"C6",IF(M36&gt;=45,"D7",IF(M36&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1523,7 +1533,7 @@
         <f>IF(COUNT(D37:J37,L37)=0,"",SUM(G37,K37,L37))</f>
       </c>
       <c r="N37" s="11">
-        <f>IF(M37="","",IF(M37&gt;=75,"A1",IF(M37&gt;=70,"B2",IF(M37&gt;=65,"B3",IF(M37&gt;=60,"C4",IF(M37&gt;=55,"C5",IF(M37&gt;=50,"C6",IF(M37&gt;=45,"D7",IF(M37&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M37="","",IF($M$3="JSS",IF(M37&gt;=80,"A",IF(M37&gt;=60,"C",IF(M37&gt;=50,"P","F"))),IF(M37&gt;=75,"A1",IF(M37&gt;=70,"B2",IF(M37&gt;=65,"B3",IF(M37&gt;=60,"C4",IF(M37&gt;=55,"C5",IF(M37&gt;=50,"C6",IF(M37&gt;=45,"D7",IF(M37&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1549,7 +1559,7 @@
         <f>IF(COUNT(D38:J38,L38)=0,"",SUM(G38,K38,L38))</f>
       </c>
       <c r="N38" s="11">
-        <f>IF(M38="","",IF(M38&gt;=75,"A1",IF(M38&gt;=70,"B2",IF(M38&gt;=65,"B3",IF(M38&gt;=60,"C4",IF(M38&gt;=55,"C5",IF(M38&gt;=50,"C6",IF(M38&gt;=45,"D7",IF(M38&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M38="","",IF($M$3="JSS",IF(M38&gt;=80,"A",IF(M38&gt;=60,"C",IF(M38&gt;=50,"P","F"))),IF(M38&gt;=75,"A1",IF(M38&gt;=70,"B2",IF(M38&gt;=65,"B3",IF(M38&gt;=60,"C4",IF(M38&gt;=55,"C5",IF(M38&gt;=50,"C6",IF(M38&gt;=45,"D7",IF(M38&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1575,7 +1585,7 @@
         <f>IF(COUNT(D39:J39,L39)=0,"",SUM(G39,K39,L39))</f>
       </c>
       <c r="N39" s="11">
-        <f>IF(M39="","",IF(M39&gt;=75,"A1",IF(M39&gt;=70,"B2",IF(M39&gt;=65,"B3",IF(M39&gt;=60,"C4",IF(M39&gt;=55,"C5",IF(M39&gt;=50,"C6",IF(M39&gt;=45,"D7",IF(M39&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M39="","",IF($M$3="JSS",IF(M39&gt;=80,"A",IF(M39&gt;=60,"C",IF(M39&gt;=50,"P","F"))),IF(M39&gt;=75,"A1",IF(M39&gt;=70,"B2",IF(M39&gt;=65,"B3",IF(M39&gt;=60,"C4",IF(M39&gt;=55,"C5",IF(M39&gt;=50,"C6",IF(M39&gt;=45,"D7",IF(M39&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1601,7 +1611,7 @@
         <f>IF(COUNT(D40:J40,L40)=0,"",SUM(G40,K40,L40))</f>
       </c>
       <c r="N40" s="11">
-        <f>IF(M40="","",IF(M40&gt;=75,"A1",IF(M40&gt;=70,"B2",IF(M40&gt;=65,"B3",IF(M40&gt;=60,"C4",IF(M40&gt;=55,"C5",IF(M40&gt;=50,"C6",IF(M40&gt;=45,"D7",IF(M40&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M40="","",IF($M$3="JSS",IF(M40&gt;=80,"A",IF(M40&gt;=60,"C",IF(M40&gt;=50,"P","F"))),IF(M40&gt;=75,"A1",IF(M40&gt;=70,"B2",IF(M40&gt;=65,"B3",IF(M40&gt;=60,"C4",IF(M40&gt;=55,"C5",IF(M40&gt;=50,"C6",IF(M40&gt;=45,"D7",IF(M40&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1627,7 +1637,7 @@
         <f>IF(COUNT(D41:J41,L41)=0,"",SUM(G41,K41,L41))</f>
       </c>
       <c r="N41" s="11">
-        <f>IF(M41="","",IF(M41&gt;=75,"A1",IF(M41&gt;=70,"B2",IF(M41&gt;=65,"B3",IF(M41&gt;=60,"C4",IF(M41&gt;=55,"C5",IF(M41&gt;=50,"C6",IF(M41&gt;=45,"D7",IF(M41&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M41="","",IF($M$3="JSS",IF(M41&gt;=80,"A",IF(M41&gt;=60,"C",IF(M41&gt;=50,"P","F"))),IF(M41&gt;=75,"A1",IF(M41&gt;=70,"B2",IF(M41&gt;=65,"B3",IF(M41&gt;=60,"C4",IF(M41&gt;=55,"C5",IF(M41&gt;=50,"C6",IF(M41&gt;=45,"D7",IF(M41&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1653,7 +1663,7 @@
         <f>IF(COUNT(D42:J42,L42)=0,"",SUM(G42,K42,L42))</f>
       </c>
       <c r="N42" s="11">
-        <f>IF(M42="","",IF(M42&gt;=75,"A1",IF(M42&gt;=70,"B2",IF(M42&gt;=65,"B3",IF(M42&gt;=60,"C4",IF(M42&gt;=55,"C5",IF(M42&gt;=50,"C6",IF(M42&gt;=45,"D7",IF(M42&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M42="","",IF($M$3="JSS",IF(M42&gt;=80,"A",IF(M42&gt;=60,"C",IF(M42&gt;=50,"P","F"))),IF(M42&gt;=75,"A1",IF(M42&gt;=70,"B2",IF(M42&gt;=65,"B3",IF(M42&gt;=60,"C4",IF(M42&gt;=55,"C5",IF(M42&gt;=50,"C6",IF(M42&gt;=45,"D7",IF(M42&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1679,7 +1689,7 @@
         <f>IF(COUNT(D43:J43,L43)=0,"",SUM(G43,K43,L43))</f>
       </c>
       <c r="N43" s="11">
-        <f>IF(M43="","",IF(M43&gt;=75,"A1",IF(M43&gt;=70,"B2",IF(M43&gt;=65,"B3",IF(M43&gt;=60,"C4",IF(M43&gt;=55,"C5",IF(M43&gt;=50,"C6",IF(M43&gt;=45,"D7",IF(M43&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M43="","",IF($M$3="JSS",IF(M43&gt;=80,"A",IF(M43&gt;=60,"C",IF(M43&gt;=50,"P","F"))),IF(M43&gt;=75,"A1",IF(M43&gt;=70,"B2",IF(M43&gt;=65,"B3",IF(M43&gt;=60,"C4",IF(M43&gt;=55,"C5",IF(M43&gt;=50,"C6",IF(M43&gt;=45,"D7",IF(M43&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1705,7 +1715,7 @@
         <f>IF(COUNT(D44:J44,L44)=0,"",SUM(G44,K44,L44))</f>
       </c>
       <c r="N44" s="11">
-        <f>IF(M44="","",IF(M44&gt;=75,"A1",IF(M44&gt;=70,"B2",IF(M44&gt;=65,"B3",IF(M44&gt;=60,"C4",IF(M44&gt;=55,"C5",IF(M44&gt;=50,"C6",IF(M44&gt;=45,"D7",IF(M44&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M44="","",IF($M$3="JSS",IF(M44&gt;=80,"A",IF(M44&gt;=60,"C",IF(M44&gt;=50,"P","F"))),IF(M44&gt;=75,"A1",IF(M44&gt;=70,"B2",IF(M44&gt;=65,"B3",IF(M44&gt;=60,"C4",IF(M44&gt;=55,"C5",IF(M44&gt;=50,"C6",IF(M44&gt;=45,"D7",IF(M44&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1731,7 +1741,7 @@
         <f>IF(COUNT(D45:J45,L45)=0,"",SUM(G45,K45,L45))</f>
       </c>
       <c r="N45" s="11">
-        <f>IF(M45="","",IF(M45&gt;=75,"A1",IF(M45&gt;=70,"B2",IF(M45&gt;=65,"B3",IF(M45&gt;=60,"C4",IF(M45&gt;=55,"C5",IF(M45&gt;=50,"C6",IF(M45&gt;=45,"D7",IF(M45&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M45="","",IF($M$3="JSS",IF(M45&gt;=80,"A",IF(M45&gt;=60,"C",IF(M45&gt;=50,"P","F"))),IF(M45&gt;=75,"A1",IF(M45&gt;=70,"B2",IF(M45&gt;=65,"B3",IF(M45&gt;=60,"C4",IF(M45&gt;=55,"C5",IF(M45&gt;=50,"C6",IF(M45&gt;=45,"D7",IF(M45&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1757,7 +1767,7 @@
         <f>IF(COUNT(D46:J46,L46)=0,"",SUM(G46,K46,L46))</f>
       </c>
       <c r="N46" s="11">
-        <f>IF(M46="","",IF(M46&gt;=75,"A1",IF(M46&gt;=70,"B2",IF(M46&gt;=65,"B3",IF(M46&gt;=60,"C4",IF(M46&gt;=55,"C5",IF(M46&gt;=50,"C6",IF(M46&gt;=45,"D7",IF(M46&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M46="","",IF($M$3="JSS",IF(M46&gt;=80,"A",IF(M46&gt;=60,"C",IF(M46&gt;=50,"P","F"))),IF(M46&gt;=75,"A1",IF(M46&gt;=70,"B2",IF(M46&gt;=65,"B3",IF(M46&gt;=60,"C4",IF(M46&gt;=55,"C5",IF(M46&gt;=50,"C6",IF(M46&gt;=45,"D7",IF(M46&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1783,7 +1793,7 @@
         <f>IF(COUNT(D47:J47,L47)=0,"",SUM(G47,K47,L47))</f>
       </c>
       <c r="N47" s="11">
-        <f>IF(M47="","",IF(M47&gt;=75,"A1",IF(M47&gt;=70,"B2",IF(M47&gt;=65,"B3",IF(M47&gt;=60,"C4",IF(M47&gt;=55,"C5",IF(M47&gt;=50,"C6",IF(M47&gt;=45,"D7",IF(M47&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M47="","",IF($M$3="JSS",IF(M47&gt;=80,"A",IF(M47&gt;=60,"C",IF(M47&gt;=50,"P","F"))),IF(M47&gt;=75,"A1",IF(M47&gt;=70,"B2",IF(M47&gt;=65,"B3",IF(M47&gt;=60,"C4",IF(M47&gt;=55,"C5",IF(M47&gt;=50,"C6",IF(M47&gt;=45,"D7",IF(M47&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1809,7 +1819,7 @@
         <f>IF(COUNT(D48:J48,L48)=0,"",SUM(G48,K48,L48))</f>
       </c>
       <c r="N48" s="11">
-        <f>IF(M48="","",IF(M48&gt;=75,"A1",IF(M48&gt;=70,"B2",IF(M48&gt;=65,"B3",IF(M48&gt;=60,"C4",IF(M48&gt;=55,"C5",IF(M48&gt;=50,"C6",IF(M48&gt;=45,"D7",IF(M48&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M48="","",IF($M$3="JSS",IF(M48&gt;=80,"A",IF(M48&gt;=60,"C",IF(M48&gt;=50,"P","F"))),IF(M48&gt;=75,"A1",IF(M48&gt;=70,"B2",IF(M48&gt;=65,"B3",IF(M48&gt;=60,"C4",IF(M48&gt;=55,"C5",IF(M48&gt;=50,"C6",IF(M48&gt;=45,"D7",IF(M48&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1835,7 +1845,7 @@
         <f>IF(COUNT(D49:J49,L49)=0,"",SUM(G49,K49,L49))</f>
       </c>
       <c r="N49" s="11">
-        <f>IF(M49="","",IF(M49&gt;=75,"A1",IF(M49&gt;=70,"B2",IF(M49&gt;=65,"B3",IF(M49&gt;=60,"C4",IF(M49&gt;=55,"C5",IF(M49&gt;=50,"C6",IF(M49&gt;=45,"D7",IF(M49&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M49="","",IF($M$3="JSS",IF(M49&gt;=80,"A",IF(M49&gt;=60,"C",IF(M49&gt;=50,"P","F"))),IF(M49&gt;=75,"A1",IF(M49&gt;=70,"B2",IF(M49&gt;=65,"B3",IF(M49&gt;=60,"C4",IF(M49&gt;=55,"C5",IF(M49&gt;=50,"C6",IF(M49&gt;=45,"D7",IF(M49&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1861,7 +1871,7 @@
         <f>IF(COUNT(D50:J50,L50)=0,"",SUM(G50,K50,L50))</f>
       </c>
       <c r="N50" s="11">
-        <f>IF(M50="","",IF(M50&gt;=75,"A1",IF(M50&gt;=70,"B2",IF(M50&gt;=65,"B3",IF(M50&gt;=60,"C4",IF(M50&gt;=55,"C5",IF(M50&gt;=50,"C6",IF(M50&gt;=45,"D7",IF(M50&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M50="","",IF($M$3="JSS",IF(M50&gt;=80,"A",IF(M50&gt;=60,"C",IF(M50&gt;=50,"P","F"))),IF(M50&gt;=75,"A1",IF(M50&gt;=70,"B2",IF(M50&gt;=65,"B3",IF(M50&gt;=60,"C4",IF(M50&gt;=55,"C5",IF(M50&gt;=50,"C6",IF(M50&gt;=45,"D7",IF(M50&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1887,7 +1897,7 @@
         <f>IF(COUNT(D51:J51,L51)=0,"",SUM(G51,K51,L51))</f>
       </c>
       <c r="N51" s="11">
-        <f>IF(M51="","",IF(M51&gt;=75,"A1",IF(M51&gt;=70,"B2",IF(M51&gt;=65,"B3",IF(M51&gt;=60,"C4",IF(M51&gt;=55,"C5",IF(M51&gt;=50,"C6",IF(M51&gt;=45,"D7",IF(M51&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M51="","",IF($M$3="JSS",IF(M51&gt;=80,"A",IF(M51&gt;=60,"C",IF(M51&gt;=50,"P","F"))),IF(M51&gt;=75,"A1",IF(M51&gt;=70,"B2",IF(M51&gt;=65,"B3",IF(M51&gt;=60,"C4",IF(M51&gt;=55,"C5",IF(M51&gt;=50,"C6",IF(M51&gt;=45,"D7",IF(M51&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1913,7 +1923,7 @@
         <f>IF(COUNT(D52:J52,L52)=0,"",SUM(G52,K52,L52))</f>
       </c>
       <c r="N52" s="11">
-        <f>IF(M52="","",IF(M52&gt;=75,"A1",IF(M52&gt;=70,"B2",IF(M52&gt;=65,"B3",IF(M52&gt;=60,"C4",IF(M52&gt;=55,"C5",IF(M52&gt;=50,"C6",IF(M52&gt;=45,"D7",IF(M52&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M52="","",IF($M$3="JSS",IF(M52&gt;=80,"A",IF(M52&gt;=60,"C",IF(M52&gt;=50,"P","F"))),IF(M52&gt;=75,"A1",IF(M52&gt;=70,"B2",IF(M52&gt;=65,"B3",IF(M52&gt;=60,"C4",IF(M52&gt;=55,"C5",IF(M52&gt;=50,"C6",IF(M52&gt;=45,"D7",IF(M52&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1939,7 +1949,7 @@
         <f>IF(COUNT(D53:J53,L53)=0,"",SUM(G53,K53,L53))</f>
       </c>
       <c r="N53" s="11">
-        <f>IF(M53="","",IF(M53&gt;=75,"A1",IF(M53&gt;=70,"B2",IF(M53&gt;=65,"B3",IF(M53&gt;=60,"C4",IF(M53&gt;=55,"C5",IF(M53&gt;=50,"C6",IF(M53&gt;=45,"D7",IF(M53&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M53="","",IF($M$3="JSS",IF(M53&gt;=80,"A",IF(M53&gt;=60,"C",IF(M53&gt;=50,"P","F"))),IF(M53&gt;=75,"A1",IF(M53&gt;=70,"B2",IF(M53&gt;=65,"B3",IF(M53&gt;=60,"C4",IF(M53&gt;=55,"C5",IF(M53&gt;=50,"C6",IF(M53&gt;=45,"D7",IF(M53&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1965,7 +1975,7 @@
         <f>IF(COUNT(D54:J54,L54)=0,"",SUM(G54,K54,L54))</f>
       </c>
       <c r="N54" s="11">
-        <f>IF(M54="","",IF(M54&gt;=75,"A1",IF(M54&gt;=70,"B2",IF(M54&gt;=65,"B3",IF(M54&gt;=60,"C4",IF(M54&gt;=55,"C5",IF(M54&gt;=50,"C6",IF(M54&gt;=45,"D7",IF(M54&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M54="","",IF($M$3="JSS",IF(M54&gt;=80,"A",IF(M54&gt;=60,"C",IF(M54&gt;=50,"P","F"))),IF(M54&gt;=75,"A1",IF(M54&gt;=70,"B2",IF(M54&gt;=65,"B3",IF(M54&gt;=60,"C4",IF(M54&gt;=55,"C5",IF(M54&gt;=50,"C6",IF(M54&gt;=45,"D7",IF(M54&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1991,7 +2001,7 @@
         <f>IF(COUNT(D55:J55,L55)=0,"",SUM(G55,K55,L55))</f>
       </c>
       <c r="N55" s="11">
-        <f>IF(M55="","",IF(M55&gt;=75,"A1",IF(M55&gt;=70,"B2",IF(M55&gt;=65,"B3",IF(M55&gt;=60,"C4",IF(M55&gt;=55,"C5",IF(M55&gt;=50,"C6",IF(M55&gt;=45,"D7",IF(M55&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M55="","",IF($M$3="JSS",IF(M55&gt;=80,"A",IF(M55&gt;=60,"C",IF(M55&gt;=50,"P","F"))),IF(M55&gt;=75,"A1",IF(M55&gt;=70,"B2",IF(M55&gt;=65,"B3",IF(M55&gt;=60,"C4",IF(M55&gt;=55,"C5",IF(M55&gt;=50,"C6",IF(M55&gt;=45,"D7",IF(M55&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2017,7 +2027,7 @@
         <f>IF(COUNT(D56:J56,L56)=0,"",SUM(G56,K56,L56))</f>
       </c>
       <c r="N56" s="11">
-        <f>IF(M56="","",IF(M56&gt;=75,"A1",IF(M56&gt;=70,"B2",IF(M56&gt;=65,"B3",IF(M56&gt;=60,"C4",IF(M56&gt;=55,"C5",IF(M56&gt;=50,"C6",IF(M56&gt;=45,"D7",IF(M56&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M56="","",IF($M$3="JSS",IF(M56&gt;=80,"A",IF(M56&gt;=60,"C",IF(M56&gt;=50,"P","F"))),IF(M56&gt;=75,"A1",IF(M56&gt;=70,"B2",IF(M56&gt;=65,"B3",IF(M56&gt;=60,"C4",IF(M56&gt;=55,"C5",IF(M56&gt;=50,"C6",IF(M56&gt;=45,"D7",IF(M56&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2043,7 +2053,7 @@
         <f>IF(COUNT(D57:J57,L57)=0,"",SUM(G57,K57,L57))</f>
       </c>
       <c r="N57" s="11">
-        <f>IF(M57="","",IF(M57&gt;=75,"A1",IF(M57&gt;=70,"B2",IF(M57&gt;=65,"B3",IF(M57&gt;=60,"C4",IF(M57&gt;=55,"C5",IF(M57&gt;=50,"C6",IF(M57&gt;=45,"D7",IF(M57&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M57="","",IF($M$3="JSS",IF(M57&gt;=80,"A",IF(M57&gt;=60,"C",IF(M57&gt;=50,"P","F"))),IF(M57&gt;=75,"A1",IF(M57&gt;=70,"B2",IF(M57&gt;=65,"B3",IF(M57&gt;=60,"C4",IF(M57&gt;=55,"C5",IF(M57&gt;=50,"C6",IF(M57&gt;=45,"D7",IF(M57&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2069,7 +2079,7 @@
         <f>IF(COUNT(D58:J58,L58)=0,"",SUM(G58,K58,L58))</f>
       </c>
       <c r="N58" s="11">
-        <f>IF(M58="","",IF(M58&gt;=75,"A1",IF(M58&gt;=70,"B2",IF(M58&gt;=65,"B3",IF(M58&gt;=60,"C4",IF(M58&gt;=55,"C5",IF(M58&gt;=50,"C6",IF(M58&gt;=45,"D7",IF(M58&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M58="","",IF($M$3="JSS",IF(M58&gt;=80,"A",IF(M58&gt;=60,"C",IF(M58&gt;=50,"P","F"))),IF(M58&gt;=75,"A1",IF(M58&gt;=70,"B2",IF(M58&gt;=65,"B3",IF(M58&gt;=60,"C4",IF(M58&gt;=55,"C5",IF(M58&gt;=50,"C6",IF(M58&gt;=45,"D7",IF(M58&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2095,7 +2105,7 @@
         <f>IF(COUNT(D59:J59,L59)=0,"",SUM(G59,K59,L59))</f>
       </c>
       <c r="N59" s="11">
-        <f>IF(M59="","",IF(M59&gt;=75,"A1",IF(M59&gt;=70,"B2",IF(M59&gt;=65,"B3",IF(M59&gt;=60,"C4",IF(M59&gt;=55,"C5",IF(M59&gt;=50,"C6",IF(M59&gt;=45,"D7",IF(M59&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M59="","",IF($M$3="JSS",IF(M59&gt;=80,"A",IF(M59&gt;=60,"C",IF(M59&gt;=50,"P","F"))),IF(M59&gt;=75,"A1",IF(M59&gt;=70,"B2",IF(M59&gt;=65,"B3",IF(M59&gt;=60,"C4",IF(M59&gt;=55,"C5",IF(M59&gt;=50,"C6",IF(M59&gt;=45,"D7",IF(M59&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2121,7 +2131,7 @@
         <f>IF(COUNT(D60:J60,L60)=0,"",SUM(G60,K60,L60))</f>
       </c>
       <c r="N60" s="11">
-        <f>IF(M60="","",IF(M60&gt;=75,"A1",IF(M60&gt;=70,"B2",IF(M60&gt;=65,"B3",IF(M60&gt;=60,"C4",IF(M60&gt;=55,"C5",IF(M60&gt;=50,"C6",IF(M60&gt;=45,"D7",IF(M60&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M60="","",IF($M$3="JSS",IF(M60&gt;=80,"A",IF(M60&gt;=60,"C",IF(M60&gt;=50,"P","F"))),IF(M60&gt;=75,"A1",IF(M60&gt;=70,"B2",IF(M60&gt;=65,"B3",IF(M60&gt;=60,"C4",IF(M60&gt;=55,"C5",IF(M60&gt;=50,"C6",IF(M60&gt;=45,"D7",IF(M60&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2147,7 +2157,7 @@
         <f>IF(COUNT(D61:J61,L61)=0,"",SUM(G61,K61,L61))</f>
       </c>
       <c r="N61" s="11">
-        <f>IF(M61="","",IF(M61&gt;=75,"A1",IF(M61&gt;=70,"B2",IF(M61&gt;=65,"B3",IF(M61&gt;=60,"C4",IF(M61&gt;=55,"C5",IF(M61&gt;=50,"C6",IF(M61&gt;=45,"D7",IF(M61&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M61="","",IF($M$3="JSS",IF(M61&gt;=80,"A",IF(M61&gt;=60,"C",IF(M61&gt;=50,"P","F"))),IF(M61&gt;=75,"A1",IF(M61&gt;=70,"B2",IF(M61&gt;=65,"B3",IF(M61&gt;=60,"C4",IF(M61&gt;=55,"C5",IF(M61&gt;=50,"C6",IF(M61&gt;=45,"D7",IF(M61&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2173,7 +2183,7 @@
         <f>IF(COUNT(D62:J62,L62)=0,"",SUM(G62,K62,L62))</f>
       </c>
       <c r="N62" s="11">
-        <f>IF(M62="","",IF(M62&gt;=75,"A1",IF(M62&gt;=70,"B2",IF(M62&gt;=65,"B3",IF(M62&gt;=60,"C4",IF(M62&gt;=55,"C5",IF(M62&gt;=50,"C6",IF(M62&gt;=45,"D7",IF(M62&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M62="","",IF($M$3="JSS",IF(M62&gt;=80,"A",IF(M62&gt;=60,"C",IF(M62&gt;=50,"P","F"))),IF(M62&gt;=75,"A1",IF(M62&gt;=70,"B2",IF(M62&gt;=65,"B3",IF(M62&gt;=60,"C4",IF(M62&gt;=55,"C5",IF(M62&gt;=50,"C6",IF(M62&gt;=45,"D7",IF(M62&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2199,7 +2209,7 @@
         <f>IF(COUNT(D63:J63,L63)=0,"",SUM(G63,K63,L63))</f>
       </c>
       <c r="N63" s="11">
-        <f>IF(M63="","",IF(M63&gt;=75,"A1",IF(M63&gt;=70,"B2",IF(M63&gt;=65,"B3",IF(M63&gt;=60,"C4",IF(M63&gt;=55,"C5",IF(M63&gt;=50,"C6",IF(M63&gt;=45,"D7",IF(M63&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M63="","",IF($M$3="JSS",IF(M63&gt;=80,"A",IF(M63&gt;=60,"C",IF(M63&gt;=50,"P","F"))),IF(M63&gt;=75,"A1",IF(M63&gt;=70,"B2",IF(M63&gt;=65,"B3",IF(M63&gt;=60,"C4",IF(M63&gt;=55,"C5",IF(M63&gt;=50,"C6",IF(M63&gt;=45,"D7",IF(M63&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2225,7 +2235,7 @@
         <f>IF(COUNT(D64:J64,L64)=0,"",SUM(G64,K64,L64))</f>
       </c>
       <c r="N64" s="11">
-        <f>IF(M64="","",IF(M64&gt;=75,"A1",IF(M64&gt;=70,"B2",IF(M64&gt;=65,"B3",IF(M64&gt;=60,"C4",IF(M64&gt;=55,"C5",IF(M64&gt;=50,"C6",IF(M64&gt;=45,"D7",IF(M64&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M64="","",IF($M$3="JSS",IF(M64&gt;=80,"A",IF(M64&gt;=60,"C",IF(M64&gt;=50,"P","F"))),IF(M64&gt;=75,"A1",IF(M64&gt;=70,"B2",IF(M64&gt;=65,"B3",IF(M64&gt;=60,"C4",IF(M64&gt;=55,"C5",IF(M64&gt;=50,"C6",IF(M64&gt;=45,"D7",IF(M64&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2251,7 +2261,7 @@
         <f>IF(COUNT(D65:J65,L65)=0,"",SUM(G65,K65,L65))</f>
       </c>
       <c r="N65" s="11">
-        <f>IF(M65="","",IF(M65&gt;=75,"A1",IF(M65&gt;=70,"B2",IF(M65&gt;=65,"B3",IF(M65&gt;=60,"C4",IF(M65&gt;=55,"C5",IF(M65&gt;=50,"C6",IF(M65&gt;=45,"D7",IF(M65&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M65="","",IF($M$3="JSS",IF(M65&gt;=80,"A",IF(M65&gt;=60,"C",IF(M65&gt;=50,"P","F"))),IF(M65&gt;=75,"A1",IF(M65&gt;=70,"B2",IF(M65&gt;=65,"B3",IF(M65&gt;=60,"C4",IF(M65&gt;=55,"C5",IF(M65&gt;=50,"C6",IF(M65&gt;=45,"D7",IF(M65&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -2277,53 +2287,81 @@
         <f>IF(COUNT(D66:J66,L66)=0,"",SUM(G66,K66,L66))</f>
       </c>
       <c r="N66" s="11">
-        <f>IF(M66="","",IF(M66&gt;=75,"A1",IF(M66&gt;=70,"B2",IF(M66&gt;=65,"B3",IF(M66&gt;=60,"C4",IF(M66&gt;=55,"C5",IF(M66&gt;=50,"C6",IF(M66&gt;=45,"D7",IF(M66&gt;=40,"E8","F9")))))))))</f>
+        <f>IF(M66="","",IF($M$3="JSS",IF(M66&gt;=80,"A",IF(M66&gt;=60,"C",IF(M66&gt;=50,"P","F"))),IF(M66&gt;=75,"A1",IF(M66&gt;=70,"B2",IF(M66&gt;=65,"B3",IF(M66&gt;=60,"C4",IF(M66&gt;=55,"C5",IF(M66&gt;=50,"C6",IF(M66&gt;=45,"D7",IF(M66&gt;=40,"E8","F9"))))))))))</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:G3"/>
-    <mergeCell ref="I3:N3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="M3:N3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="E4:G4"/>
     <mergeCell ref="I4:N4"/>
     <mergeCell ref="A5:N5"/>
   </mergeCells>
-  <dataValidations count="8">
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 15." sqref="D10:D66">
+  <dataValidations count="15">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 10." sqref="D10:D66">
       <formula1>0</formula1>
-      <formula2>15</formula2>
+      <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 15." sqref="D7:D66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 10." sqref="D7:D66">
       <formula1>0</formula1>
-      <formula2>15</formula2>
+      <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 5." sqref="E10:F66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 2." sqref="E10:E66">
       <formula1>0</formula1>
-      <formula2>5</formula2>
+      <formula2>2</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 5." sqref="E7:F66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 2." sqref="E7:E66">
       <formula1>0</formula1>
-      <formula2>5</formula2>
+      <formula2>2</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 5." sqref="H10:J66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 3." sqref="F10:F66">
       <formula1>0</formula1>
-      <formula2>5</formula2>
+      <formula2>3</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 5." sqref="H7:J66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 3." sqref="F7:F66">
       <formula1>0</formula1>
-      <formula2>5</formula2>
+      <formula2>3</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 60." sqref="L10:L66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 10." sqref="H10:H66">
       <formula1>0</formula1>
-      <formula2>60</formula2>
+      <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 60." sqref="L7:L66">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 10." sqref="H7:H66">
       <formula1>0</formula1>
-      <formula2>60</formula2>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 3." sqref="I10:I66">
+      <formula1>0</formula1>
+      <formula2>3</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 3." sqref="I7:I66">
+      <formula1>0</formula1>
+      <formula2>3</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 2." sqref="J10:J66">
+      <formula1>0</formula1>
+      <formula2>2</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 2." sqref="J7:J66">
+      <formula1>0</formula1>
+      <formula2>2</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 70." sqref="L10:L66">
+      <formula1>0</formula1>
+      <formula2>70</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Score out of range" error="Enter a number from 0 to 70." sqref="L7:L66">
+      <formula1>0</formula1>
+      <formula2>70</formula2>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Level" error="Choose JSS or SSS." sqref="M3">
+      <formula1>"SSS,JSS"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>

</xml_diff>